<commit_message>
Add SOH report for 2026-10-21
</commit_message>
<xml_diff>
--- a/reports/SOH_20_10_2026.xlsx
+++ b/reports/SOH_20_10_2026.xlsx
@@ -965,7 +965,7 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>1</v>
@@ -1749,7 +1749,7 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>1407</v>
+        <v>1406</v>
       </c>
       <c r="E47" s="3" t="n">
         <v>1195</v>
@@ -4713,7 +4713,7 @@
         </is>
       </c>
       <c r="D153" s="2" t="n">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="E153" s="3" t="n">
         <v>1</v>
@@ -4825,7 +4825,7 @@
         </is>
       </c>
       <c r="D157" s="2" t="n">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="E157" s="3" t="n">
         <v>26000</v>
@@ -6713,7 +6713,7 @@
         </is>
       </c>
       <c r="D227" s="2" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E227" s="3" t="n">
         <v>1</v>
@@ -9471,24 +9471,24 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>9333527490599</t>
+          <t>9333527490506</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>BB0178</t>
+          <t>BB0170</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>BAX TILE &amp; GROUT BRUSH</t>
+          <t>BAX SQUEEZE SPONGE MOP</t>
         </is>
       </c>
       <c r="D327" s="2" t="n">
-        <v>426</v>
+        <v>141</v>
       </c>
       <c r="E327" s="3" t="n">
-        <v>12666</v>
+        <v>33956</v>
       </c>
       <c r="F327" t="inlineStr">
         <is>
@@ -9499,24 +9499,24 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>9333527490506</t>
+          <t>9333527490599</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>BB0170</t>
+          <t>BB0178</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>BAX SQUEEZE SPONGE MOP</t>
+          <t>BAX TILE &amp; GROUT BRUSH</t>
         </is>
       </c>
       <c r="D328" s="2" t="n">
-        <v>141</v>
+        <v>426</v>
       </c>
       <c r="E328" s="3" t="n">
-        <v>33956</v>
+        <v>12666</v>
       </c>
       <c r="F328" t="inlineStr">
         <is>
@@ -32355,24 +32355,24 @@
     <row r="1144">
       <c r="A1144" t="inlineStr">
         <is>
-          <t>9333527037817</t>
+          <t>9333527582744</t>
         </is>
       </c>
       <c r="B1144" t="inlineStr">
         <is>
-          <t>AG0222</t>
+          <t>SG0474</t>
         </is>
       </c>
       <c r="C1144" t="inlineStr">
         <is>
-          <t>NYLON BATH BALL 30GM 3PK TUB</t>
+          <t>NOVELTY ERASER 6 ASSORTED</t>
         </is>
       </c>
       <c r="D1144" s="2" t="n">
-        <v>180</v>
+        <v>256</v>
       </c>
       <c r="E1144" s="3" t="n">
-        <v>11027</v>
+        <v>7975</v>
       </c>
       <c r="F1144" t="inlineStr">
         <is>
@@ -32383,24 +32383,24 @@
     <row r="1145">
       <c r="A1145" t="inlineStr">
         <is>
-          <t>4894158158555</t>
+          <t>9333527779809</t>
         </is>
       </c>
       <c r="B1145" t="inlineStr">
         <is>
-          <t>XM6877</t>
+          <t>XD0000098</t>
         </is>
       </c>
       <c r="C1145" t="inlineStr">
         <is>
-          <t>NUTBELL HANGER VELVET BOW 8cm Asst</t>
+          <t>NUTBELL HANGER CANDYSTRIPE BOW 20cm Asst</t>
         </is>
       </c>
       <c r="D1145" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E1145" s="3" t="n">
-        <v>17096</v>
+        <v>31943</v>
       </c>
       <c r="F1145" t="inlineStr">
         <is>
@@ -32411,24 +32411,24 @@
     <row r="1146">
       <c r="A1146" t="inlineStr">
         <is>
-          <t>9333527779809</t>
+          <t>4894158158555</t>
         </is>
       </c>
       <c r="B1146" t="inlineStr">
         <is>
-          <t>XD0000098</t>
+          <t>XM6877</t>
         </is>
       </c>
       <c r="C1146" t="inlineStr">
         <is>
-          <t>NUTBELL HANGER CANDYSTRIPE BOW 20cm Asst</t>
+          <t>NUTBELL HANGER VELVET BOW 8cm Asst</t>
         </is>
       </c>
       <c r="D1146" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E1146" s="3" t="n">
-        <v>31943</v>
+        <v>17096</v>
       </c>
       <c r="F1146" t="inlineStr">
         <is>
@@ -32439,24 +32439,24 @@
     <row r="1147">
       <c r="A1147" t="inlineStr">
         <is>
-          <t>9333527665270</t>
+          <t>9333527037817</t>
         </is>
       </c>
       <c r="B1147" t="inlineStr">
         <is>
-          <t>SC0469</t>
+          <t>AG0222</t>
         </is>
       </c>
       <c r="C1147" t="inlineStr">
         <is>
-          <t>OCCASSIONS BAG 26X32.4CM 4ASST</t>
+          <t>NYLON BATH BALL 30GM 3PK TUB</t>
         </is>
       </c>
       <c r="D1147" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="E1147" s="3" t="n">
-        <v>6064</v>
+        <v>11027</v>
       </c>
       <c r="F1147" t="inlineStr">
         <is>
@@ -32467,24 +32467,24 @@
     <row r="1148">
       <c r="A1148" t="inlineStr">
         <is>
-          <t>9333527582744</t>
+          <t>9333527665270</t>
         </is>
       </c>
       <c r="B1148" t="inlineStr">
         <is>
-          <t>SG0474</t>
+          <t>SC0469</t>
         </is>
       </c>
       <c r="C1148" t="inlineStr">
         <is>
-          <t>NOVELTY ERASER 6 ASSORTED</t>
+          <t>OCCASSIONS BAG 26X32.4CM 4ASST</t>
         </is>
       </c>
       <c r="D1148" s="2" t="n">
-        <v>256</v>
+        <v>0</v>
       </c>
       <c r="E1148" s="3" t="n">
-        <v>7975</v>
+        <v>6064</v>
       </c>
       <c r="F1148" t="inlineStr">
         <is>
@@ -40797,7 +40797,7 @@
         </is>
       </c>
       <c r="D1445" s="2" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E1445" s="3" t="n">
         <v>13734</v>

</xml_diff>